<commit_message>
Agregar pestaña Grupos y usar DNI como tercer campo del titular.
El Excel de grupos acepta Nombre|mail|DNI sin exigir teléfono, y los titulares se listan aparte de Personas.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/scripts/ejemplo_grupos_padre_chicos.xlsx
+++ b/scripts/ejemplo_grupos_padre_chicos.xlsx
@@ -442,7 +442,7 @@
         <v>Hijo/a</v>
       </c>
       <c r="G2" t="str">
-        <v>Martín García | martin.garcia@mail.com | 1144556677</v>
+        <v>Martín García | martin.garcia@mail.com | 30111222</v>
       </c>
     </row>
     <row r="3">
@@ -465,7 +465,7 @@
         <v>Hijo/a</v>
       </c>
       <c r="G3" t="str">
-        <v>Martín García | martin.garcia@mail.com | 1144556677</v>
+        <v>Martín García | martin.garcia@mail.com | 30111222</v>
       </c>
     </row>
     <row r="4">
@@ -488,7 +488,7 @@
         <v>Hijo/a</v>
       </c>
       <c r="G4" t="str">
-        <v>Ana López | ana.lopez@mail.com | 1166778899</v>
+        <v>Ana López | 28999888</v>
       </c>
     </row>
     <row r="5">
@@ -511,7 +511,7 @@
         <v>Hijo/a</v>
       </c>
       <c r="G5" t="str">
-        <v>Ana López | ana.lopez@mail.com | 1166778899</v>
+        <v>Ana López | 28999888</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         <v>Hijo/a</v>
       </c>
       <c r="G6" t="str">
-        <v>Ana López | ana.lopez@mail.com | 1166778899</v>
+        <v>Ana López | 28999888</v>
       </c>
     </row>
   </sheetData>

</xml_diff>